<commit_message>
fix bug in gto grad eval and add more benchmarks
</commit_message>
<xml_diff>
--- a/benchmarks_tests/FINAL_Benchmarks_for_paper/PyFock_CPU_vs_GPU_SAO.xlsx
+++ b/benchmarks_tests/FINAL_Benchmarks_for_paper/PyFock_CPU_vs_GPU_SAO.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/manas/Documents/PyFock/benchmarks_tests/FINAL_Benchmarks_for_paper/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2223E185-8A2B-1E40-9DD5-7526C8F73BF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A3A7DA1-97DE-AB43-86E7-FBFFE76F131F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="640" yWindow="3800" windowWidth="27640" windowHeight="16460" xr2:uid="{0352C87C-B4A4-4D4C-883B-F1396BEEBBFA}"/>
+    <workbookView xWindow="640" yWindow="1140" windowWidth="27640" windowHeight="16460" xr2:uid="{0352C87C-B4A4-4D4C-883B-F1396BEEBBFA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="23">
   <si>
     <t>PyFock CPU vs GPU</t>
   </si>
@@ -77,27 +77,6 @@
     <t>GPU</t>
   </si>
   <si>
-    <t>Comparison Total</t>
-  </si>
-  <si>
-    <t>Total time/iter (s) GPU</t>
-  </si>
-  <si>
-    <t>Total time/iter (s) CPU</t>
-  </si>
-  <si>
-    <t>XC / iter (s) (CPU)</t>
-  </si>
-  <si>
-    <t>XC / iter (s) (GPU)</t>
-  </si>
-  <si>
-    <t>J  / iter (s) (CPU)</t>
-  </si>
-  <si>
-    <t>J  / iter (s) (GPU)</t>
-  </si>
-  <si>
     <t>Cholesky off</t>
   </si>
   <si>
@@ -111,13 +90,28 @@
   </si>
   <si>
     <t>CPU 4 cores</t>
+  </si>
+  <si>
+    <t>CPU 32 cores</t>
+  </si>
+  <si>
+    <t>PyFock</t>
+  </si>
+  <si>
+    <t>PySCF</t>
+  </si>
+  <si>
+    <t>Grids time (s)</t>
+  </si>
+  <si>
+    <t>Tot-grids (s)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -141,13 +135,6 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
@@ -177,7 +164,9 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,7 +501,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB30E5BC-ACB8-5342-8560-2CBC0237DCD6}">
-  <dimension ref="A1:I41"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="21.6640625" customWidth="1"/>
@@ -535,7 +524,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.2">
@@ -543,10 +532,10 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="C3" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
@@ -554,7 +543,7 @@
         <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
@@ -594,18 +583,6 @@
       <c r="D6" s="2"/>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
-      <c r="G6" t="e">
-        <f>C6/F6</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H6" t="e">
-        <f>D6/F6</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I6" t="e">
-        <f>E6/F6</f>
-        <v>#DIV/0!</v>
-      </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A7">
@@ -618,18 +595,6 @@
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
-      <c r="G7" t="e">
-        <f t="shared" ref="G7:G14" si="0">C7/F7</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="H7" t="e">
-        <f t="shared" ref="H7:H14" si="1">D7/F7</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="I7" t="e">
-        <f t="shared" ref="I7:I14" si="2">E7/F7</f>
-        <v>#DIV/0!</v>
-      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A8">
@@ -651,15 +616,15 @@
         <v>13</v>
       </c>
       <c r="G8">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="G8:G14" si="0">C8/F8</f>
         <v>0.18307692307692308</v>
       </c>
       <c r="H8">
-        <f t="shared" si="1"/>
+        <f t="shared" ref="H8:H14" si="1">D8/F8</f>
         <v>5.2307692307692312E-2</v>
       </c>
       <c r="I8">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="I8:I14" si="2">E8/F8</f>
         <v>8.1538461538461546E-2</v>
       </c>
     </row>
@@ -855,9 +820,14 @@
         <v>1.5685714285714287</v>
       </c>
     </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A16" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.2">
@@ -1157,100 +1127,795 @@
         <v>21.30857142857143</v>
       </c>
     </row>
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A29" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A30" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A31" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I31" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A32" s="1" t="s">
+      <c r="A32" s="3">
+        <v>1</v>
+      </c>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A33" s="3">
+        <v>5</v>
+      </c>
+      <c r="B33">
+        <v>120</v>
+      </c>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A34" s="3">
+        <v>10</v>
+      </c>
+      <c r="B34">
+        <v>240</v>
+      </c>
+      <c r="C34" s="2">
+        <v>6.14</v>
+      </c>
+      <c r="D34" s="2">
+        <v>0.69</v>
+      </c>
+      <c r="E34" s="2">
+        <v>3.32</v>
+      </c>
+      <c r="F34" s="2">
         <v>13</v>
       </c>
-    </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A33" s="1" t="s">
+      <c r="G34" s="3">
+        <f t="shared" ref="G34:G40" si="5">C34/$F34</f>
+        <v>0.47230769230769226</v>
+      </c>
+      <c r="H34" s="3">
+        <f t="shared" ref="H34:H40" si="6">D34/$F34</f>
+        <v>5.307692307692307E-2</v>
+      </c>
+      <c r="I34" s="3">
+        <f t="shared" ref="I34:I40" si="7">E34/$F34</f>
+        <v>0.25538461538461538</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A35" s="3">
+        <v>20</v>
+      </c>
+      <c r="B35">
+        <v>480</v>
+      </c>
+      <c r="C35" s="2">
+        <v>13.62</v>
+      </c>
+      <c r="D35" s="2">
+        <v>2.37</v>
+      </c>
+      <c r="E35" s="2">
+        <v>7.25</v>
+      </c>
+      <c r="F35" s="2">
+        <v>13</v>
+      </c>
+      <c r="G35" s="3">
+        <f t="shared" si="5"/>
+        <v>1.0476923076923077</v>
+      </c>
+      <c r="H35" s="3">
+        <f t="shared" si="6"/>
+        <v>0.18230769230769231</v>
+      </c>
+      <c r="I35" s="3">
+        <f t="shared" si="7"/>
+        <v>0.55769230769230771</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A36" s="3">
+        <v>32</v>
+      </c>
+      <c r="B36">
+        <v>768</v>
+      </c>
+      <c r="C36" s="2">
+        <v>29.76</v>
+      </c>
+      <c r="D36" s="2">
+        <v>7.07</v>
+      </c>
+      <c r="E36" s="2">
+        <v>12.76</v>
+      </c>
+      <c r="F36" s="2">
+        <v>15</v>
+      </c>
+      <c r="G36" s="3">
+        <f t="shared" si="5"/>
+        <v>1.9840000000000002</v>
+      </c>
+      <c r="H36" s="3">
+        <f t="shared" si="6"/>
+        <v>0.47133333333333333</v>
+      </c>
+      <c r="I36" s="3">
+        <f t="shared" si="7"/>
+        <v>0.85066666666666668</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A37" s="3">
+        <v>47</v>
+      </c>
+      <c r="B37">
+        <v>1128</v>
+      </c>
+      <c r="C37" s="2">
+        <v>58.86</v>
+      </c>
+      <c r="D37" s="2">
+        <v>17.34</v>
+      </c>
+      <c r="E37" s="2">
+        <v>20.74</v>
+      </c>
+      <c r="F37" s="2">
+        <v>16</v>
+      </c>
+      <c r="G37" s="3">
+        <f t="shared" si="5"/>
+        <v>3.67875</v>
+      </c>
+      <c r="H37" s="3">
+        <f t="shared" si="6"/>
+        <v>1.08375</v>
+      </c>
+      <c r="I37" s="3">
+        <f t="shared" si="7"/>
+        <v>1.2962499999999999</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A38" s="3">
+        <v>76</v>
+      </c>
+      <c r="B38">
+        <v>1824</v>
+      </c>
+      <c r="C38" s="2">
+        <v>152.24</v>
+      </c>
+      <c r="D38" s="2">
+        <v>51.22</v>
+      </c>
+      <c r="E38" s="2">
+        <v>41.38</v>
+      </c>
+      <c r="F38" s="2">
+        <v>17</v>
+      </c>
+      <c r="G38" s="3">
+        <f t="shared" si="5"/>
+        <v>8.9552941176470586</v>
+      </c>
+      <c r="H38" s="3">
+        <f t="shared" si="6"/>
+        <v>3.012941176470588</v>
+      </c>
+      <c r="I38" s="3">
+        <f t="shared" si="7"/>
+        <v>2.4341176470588235</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A39" s="3">
+        <v>100</v>
+      </c>
+      <c r="B39">
+        <v>2400</v>
+      </c>
+      <c r="C39" s="2">
+        <v>230.54</v>
+      </c>
+      <c r="D39" s="2">
+        <v>67.290000000000006</v>
+      </c>
+      <c r="E39" s="2">
+        <v>60.2</v>
+      </c>
+      <c r="F39" s="2">
+        <v>16</v>
+      </c>
+      <c r="G39" s="3">
+        <f t="shared" si="5"/>
+        <v>14.40875</v>
+      </c>
+      <c r="H39" s="3">
+        <f t="shared" si="6"/>
+        <v>4.2056250000000004</v>
+      </c>
+      <c r="I39" s="3">
+        <f t="shared" si="7"/>
+        <v>3.7625000000000002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A40" s="3">
+        <v>139</v>
+      </c>
+      <c r="B40">
+        <v>3336</v>
+      </c>
+      <c r="C40" s="2">
+        <v>403.04</v>
+      </c>
+      <c r="D40" s="2">
+        <v>119.59</v>
+      </c>
+      <c r="E40" s="2">
+        <v>90.46</v>
+      </c>
+      <c r="F40" s="2">
+        <v>14</v>
+      </c>
+      <c r="G40" s="3">
+        <f t="shared" si="5"/>
+        <v>28.78857142857143</v>
+      </c>
+      <c r="H40" s="3">
+        <f t="shared" si="6"/>
+        <v>8.5421428571428581</v>
+      </c>
+      <c r="I40" s="3">
+        <f t="shared" si="7"/>
+        <v>6.4614285714285709</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A43" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A44" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A45" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B45" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D33" s="1" t="s">
+      <c r="C45" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H45" s="1"/>
+      <c r="I45" s="1"/>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A46" s="3">
+        <v>1</v>
+      </c>
+      <c r="C46" s="3"/>
+      <c r="D46" s="3"/>
+      <c r="E46" s="3"/>
+      <c r="F46" s="3"/>
+      <c r="G46" s="3"/>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3"/>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A47" s="3">
+        <v>5</v>
+      </c>
+      <c r="B47">
+        <v>120</v>
+      </c>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="G47" s="3"/>
+      <c r="H47" s="3"/>
+      <c r="I47" s="3"/>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A48" s="3">
+        <v>10</v>
+      </c>
+      <c r="B48">
+        <v>240</v>
+      </c>
+      <c r="C48" s="2">
+        <v>16.036005578003799</v>
+      </c>
+      <c r="D48" s="4">
+        <v>0.83</v>
+      </c>
+      <c r="E48" s="2">
+        <f t="shared" ref="E48:E54" si="8">C48-D48</f>
+        <v>15.206005578003799</v>
+      </c>
+      <c r="F48" s="2">
+        <v>12</v>
+      </c>
+      <c r="G48" s="3">
+        <f>E48/$F48</f>
+        <v>1.2671671315003166</v>
+      </c>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A49" s="3">
+        <v>20</v>
+      </c>
+      <c r="B49">
+        <v>480</v>
+      </c>
+      <c r="C49" s="2">
+        <v>75.564415230008294</v>
+      </c>
+      <c r="D49" s="4">
+        <v>3.34</v>
+      </c>
+      <c r="E49" s="2">
+        <f t="shared" si="8"/>
+        <v>72.22441523000829</v>
+      </c>
+      <c r="F49" s="2">
         <v>15</v>
       </c>
-      <c r="E33" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F33" s="1" t="s">
+      <c r="G49" s="3">
+        <f t="shared" ref="G49:G54" si="9">E49/$F49</f>
+        <v>4.8149610153338864</v>
+      </c>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A50" s="3">
+        <v>32</v>
+      </c>
+      <c r="B50">
+        <v>768</v>
+      </c>
+      <c r="C50" s="2">
+        <v>185.093209467013</v>
+      </c>
+      <c r="D50" s="4">
+        <v>9.19</v>
+      </c>
+      <c r="E50" s="2">
+        <f t="shared" si="8"/>
+        <v>175.903209467013</v>
+      </c>
+      <c r="F50" s="2">
+        <v>15</v>
+      </c>
+      <c r="G50" s="3">
+        <f t="shared" si="9"/>
+        <v>11.7268806311342</v>
+      </c>
+      <c r="H50" s="3"/>
+      <c r="I50" s="3"/>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A51" s="3">
+        <v>47</v>
+      </c>
+      <c r="B51">
+        <v>1128</v>
+      </c>
+      <c r="C51" s="2">
+        <v>383.57993331502001</v>
+      </c>
+      <c r="D51" s="4">
+        <v>22.52</v>
+      </c>
+      <c r="E51" s="2">
+        <f>C51-D51</f>
+        <v>361.05993331502003</v>
+      </c>
+      <c r="F51" s="2">
+        <v>15</v>
+      </c>
+      <c r="G51" s="3">
+        <f t="shared" si="9"/>
+        <v>24.070662221001335</v>
+      </c>
+      <c r="H51" s="3"/>
+      <c r="I51" s="3"/>
+    </row>
+    <row r="52" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A52" s="3">
+        <v>76</v>
+      </c>
+      <c r="B52">
+        <v>1824</v>
+      </c>
+      <c r="C52" s="2">
+        <v>1018.329558144</v>
+      </c>
+      <c r="D52" s="4">
+        <v>79.13</v>
+      </c>
+      <c r="E52" s="2">
+        <f t="shared" si="8"/>
+        <v>939.19955814399998</v>
+      </c>
+      <c r="F52" s="2">
+        <v>15</v>
+      </c>
+      <c r="G52" s="3">
+        <f t="shared" si="9"/>
+        <v>62.613303876266663</v>
+      </c>
+      <c r="H52" s="3"/>
+      <c r="I52" s="3"/>
+    </row>
+    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A53" s="3">
+        <v>100</v>
+      </c>
+      <c r="B53">
+        <v>2400</v>
+      </c>
+      <c r="C53" s="2">
+        <v>2269.11304578199</v>
+      </c>
+      <c r="D53" s="4">
+        <v>167.72</v>
+      </c>
+      <c r="E53" s="2">
+        <f t="shared" si="8"/>
+        <v>2101.3930457819902</v>
+      </c>
+      <c r="F53" s="2">
         <v>18</v>
       </c>
-      <c r="G33" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H33" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A34">
+      <c r="G53" s="3">
+        <f t="shared" si="9"/>
+        <v>116.74405809899946</v>
+      </c>
+      <c r="H53" s="3"/>
+      <c r="I53" s="3"/>
+    </row>
+    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A54" s="3">
+        <v>139</v>
+      </c>
+      <c r="B54">
+        <v>3336</v>
+      </c>
+      <c r="C54" s="2">
+        <v>3856.7203670029899</v>
+      </c>
+      <c r="D54" s="4">
+        <v>424.55</v>
+      </c>
+      <c r="E54" s="2">
+        <f t="shared" si="8"/>
+        <v>3432.1703670029897</v>
+      </c>
+      <c r="F54" s="2">
+        <v>15</v>
+      </c>
+      <c r="G54" s="3">
+        <f t="shared" si="9"/>
+        <v>228.81135780019932</v>
+      </c>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3"/>
+    </row>
+    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A56" s="1" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A57" s="1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A58" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C58" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B34">
+      <c r="D58" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G58" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H58" s="1"/>
+      <c r="I58" s="1"/>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A59" s="3">
+        <v>1</v>
+      </c>
+      <c r="C59" s="3"/>
+      <c r="D59" s="3"/>
+      <c r="E59" s="3"/>
+      <c r="F59" s="3"/>
+      <c r="G59" s="3"/>
+      <c r="H59" s="3"/>
+      <c r="I59" s="3"/>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A60" s="3">
+        <v>5</v>
+      </c>
+      <c r="B60">
         <v>120</v>
       </c>
-    </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A35">
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+      <c r="G60" s="3"/>
+      <c r="H60" s="3"/>
+      <c r="I60" s="3"/>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A61" s="3">
         <v>10</v>
       </c>
-      <c r="B35">
+      <c r="B61">
         <v>240</v>
       </c>
-    </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A36">
+      <c r="C61" s="2">
+        <v>6.6409583720378498</v>
+      </c>
+      <c r="D61" s="2">
+        <v>0.4</v>
+      </c>
+      <c r="E61" s="2">
+        <f>C61-D61</f>
+        <v>6.2409583720378494</v>
+      </c>
+      <c r="F61" s="2">
+        <v>12</v>
+      </c>
+      <c r="G61" s="3">
+        <f>C61/$F61</f>
+        <v>0.55341319766982078</v>
+      </c>
+      <c r="H61" s="3"/>
+      <c r="I61" s="3"/>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A62" s="3">
         <v>20</v>
       </c>
-      <c r="B36">
+      <c r="B62">
         <v>480</v>
       </c>
-    </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A37">
+      <c r="C62" s="2">
+        <v>27.854180095950099</v>
+      </c>
+      <c r="D62" s="2">
+        <v>1.21</v>
+      </c>
+      <c r="E62" s="2">
+        <f t="shared" ref="E62:E66" si="10">C62-D62</f>
+        <v>26.644180095950098</v>
+      </c>
+      <c r="F62" s="2">
+        <v>15</v>
+      </c>
+      <c r="G62" s="3">
+        <f t="shared" ref="G62:G67" si="11">C62/$F62</f>
+        <v>1.8569453397300066</v>
+      </c>
+      <c r="H62" s="3"/>
+      <c r="I62" s="3"/>
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A63" s="3">
         <v>32</v>
       </c>
-      <c r="B37">
+      <c r="B63">
         <v>768</v>
       </c>
-    </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A38">
+      <c r="C63" s="2">
+        <v>45.117813314893198</v>
+      </c>
+      <c r="D63" s="2">
+        <v>2.62</v>
+      </c>
+      <c r="E63" s="2">
+        <f t="shared" si="10"/>
+        <v>42.4978133148932</v>
+      </c>
+      <c r="F63" s="2">
+        <v>15</v>
+      </c>
+      <c r="G63" s="3">
+        <f t="shared" si="11"/>
+        <v>3.00785422099288</v>
+      </c>
+      <c r="H63" s="3"/>
+      <c r="I63" s="3"/>
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A64" s="3">
         <v>47</v>
       </c>
-      <c r="B38">
+      <c r="B64">
         <v>1128</v>
       </c>
-    </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A39">
+      <c r="C64" s="2">
+        <v>79.639858498936505</v>
+      </c>
+      <c r="D64" s="2">
+        <v>6.21</v>
+      </c>
+      <c r="E64" s="2">
+        <f t="shared" si="10"/>
+        <v>73.429858498936511</v>
+      </c>
+      <c r="F64" s="2">
+        <v>15</v>
+      </c>
+      <c r="G64" s="3">
+        <f t="shared" si="11"/>
+        <v>5.3093238999291001</v>
+      </c>
+      <c r="H64" s="3"/>
+      <c r="I64" s="3"/>
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A65" s="3">
         <v>76</v>
       </c>
-      <c r="B39">
+      <c r="B65">
         <v>1824</v>
       </c>
-    </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A40">
+      <c r="C65" s="2">
+        <v>193.031947857001</v>
+      </c>
+      <c r="D65" s="2">
+        <v>19.239999999999998</v>
+      </c>
+      <c r="E65" s="2">
+        <f t="shared" si="10"/>
+        <v>173.79194785700099</v>
+      </c>
+      <c r="F65" s="2">
+        <v>15</v>
+      </c>
+      <c r="G65" s="3">
+        <f t="shared" si="11"/>
+        <v>12.868796523800066</v>
+      </c>
+      <c r="H65" s="3"/>
+      <c r="I65" s="3"/>
+    </row>
+    <row r="66" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A66" s="3">
         <v>100</v>
       </c>
-      <c r="B40">
+      <c r="B66">
         <v>2400</v>
       </c>
-    </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A41">
+      <c r="C66" s="2">
+        <v>417.932956116041</v>
+      </c>
+      <c r="D66" s="2">
+        <v>39.72</v>
+      </c>
+      <c r="E66" s="2">
+        <f t="shared" si="10"/>
+        <v>378.21295611604103</v>
+      </c>
+      <c r="F66" s="2">
+        <v>18</v>
+      </c>
+      <c r="G66" s="3">
+        <f t="shared" si="11"/>
+        <v>23.218497562002277</v>
+      </c>
+      <c r="H66" s="3"/>
+      <c r="I66" s="3"/>
+    </row>
+    <row r="67" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="A67" s="3">
         <v>139</v>
       </c>
-      <c r="B41">
+      <c r="B67">
         <v>3336</v>
       </c>
+      <c r="C67" s="2">
+        <v>681.56127504497999</v>
+      </c>
+      <c r="D67" s="2">
+        <v>95.43</v>
+      </c>
+      <c r="E67" s="2">
+        <f>C67-D67</f>
+        <v>586.13127504497993</v>
+      </c>
+      <c r="F67" s="2">
+        <v>15</v>
+      </c>
+      <c r="G67" s="3">
+        <f t="shared" si="11"/>
+        <v>45.437418336332001</v>
+      </c>
+      <c r="H67" s="3"/>
+      <c r="I67" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>